<commit_message>
GUI Design advanced, chose colors, button enabling or disabling, ... Also, CLI portion pretty much handled, updates run correctly (at least for 9200 CX 12 Port, all the way from installing, checking, and cleaning files. Still have to do code cleaning and beautifying for the CLI portion.
</commit_message>
<xml_diff>
--- a/LAN_Network_Devices.xlsx
+++ b/LAN_Network_Devices.xlsx
@@ -81,7 +81,14 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="50">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -92,6 +99,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -106,6 +127,27 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -113,6 +155,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -120,6 +176,27 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -127,6 +204,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -148,6 +232,104 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.7998901333658864"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.5998718222602009"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.7998901333658864"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.5998718222602009"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.7998901333658864"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="5" tint="0.5998718222602009"/>
         </patternFill>
       </fill>
@@ -155,13 +337,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.7998901333658864"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="4" tint="0.5998718222602009"/>
         </patternFill>
       </fill>
@@ -172,6 +347,108 @@
           <bgColor theme="4" tint="0.7998901333658864"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.7998901333658864"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.5998718222602009"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <border>
@@ -233,6 +510,24 @@
         <horizontal style="thin">
           <color indexed="64"/>
         </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -332,18 +627,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1_2" displayName="Table1_2" ref="A1:I6" headerRowCount="1" totalsRowShown="0" headerRowDxfId="17">
-  <autoFilter ref="A1:I6"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1_2" displayName="Table1_2" ref="A1:N8" headerRowCount="1" totalsRowShown="0" headerRowDxfId="49">
+  <autoFilter ref="A1:N8"/>
+  <tableColumns count="14">
     <tableColumn id="1" name="Hostname"/>
     <tableColumn id="2" name="Model"/>
     <tableColumn id="3" name="OOBM IP Address"/>
     <tableColumn id="4" name="Current IOS Version"/>
     <tableColumn id="5" name="Recommended IOS Version"/>
-    <tableColumn id="6" name="Status" dataDxfId="16"/>
-    <tableColumn id="7" name="Enough Flash Space" dataDxfId="15"/>
-    <tableColumn id="9" name="Update IOS File Present" dataDxfId="14"/>
-    <tableColumn id="8" name="Needs Update" dataDxfId="13"/>
+    <tableColumn id="6" name="Status" dataDxfId="48"/>
+    <tableColumn id="10" name="Auth Status" dataDxfId="47"/>
+    <tableColumn id="7" name="Enough Flash Space" dataDxfId="46"/>
+    <tableColumn id="9" name="Update IOS File Present" dataDxfId="45"/>
+    <tableColumn id="8" name="Needs Update" dataDxfId="44"/>
+    <tableColumn id="12" name="Transfer Result" dataDxfId="43"/>
+    <tableColumn id="11" name="Install Status" dataDxfId="42"/>
+    <tableColumn id="13" name="Update Result" dataDxfId="41"/>
+    <tableColumn id="14" name="Cleaned Inactive" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -529,7 +829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="14.140625" customWidth="1" min="1" max="1"/>
@@ -538,9 +838,14 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="10.42578125" customWidth="1" min="6" max="6"/>
-    <col width="21.5703125" customWidth="1" min="7" max="7"/>
-    <col width="25.42578125" customWidth="1" min="8" max="8"/>
-    <col width="16.28515625" customWidth="1" min="9" max="9"/>
+    <col width="13.5703125" customWidth="1" min="7" max="7"/>
+    <col width="21.5703125" customWidth="1" min="8" max="8"/>
+    <col width="25.42578125" customWidth="1" min="9" max="9"/>
+    <col width="16.28515625" customWidth="1" min="10" max="10"/>
+    <col width="18.140625" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="17.5703125" customWidth="1" min="13" max="13"/>
+    <col width="19.28515625" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -576,17 +881,42 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
+          <t>Auth Status</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>Enough Flash Space</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Update IOS File Present</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Needs Update</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Transfer Result</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Install Status</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>Update Result</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>Cleaned Inactive</t>
         </is>
       </c>
     </row>
@@ -623,17 +953,42 @@
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
+          <t>AUTH_OK</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="H2" s="1" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="I2" s="1" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>YES</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>NOT_ATTEMPTED</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -670,7 +1025,7 @@
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>AUTH_OK</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
@@ -680,34 +1035,59 @@
       </c>
       <c r="I3" s="1" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
           <t>NO</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>NOT_ATTEMPTED</t>
+        </is>
+      </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="4" ht="13.9" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>SW3</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>C8KV</t>
+          <t>C9200</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>10.17.1.11</t>
+          <t>10.17.1.15</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>17.13.1a</t>
+          <t>17.12.6</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>17.15.04c</t>
+          <t>17.12.05</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
@@ -717,44 +1097,69 @@
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
+          <t>AUTH_OK</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="I4" s="1" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="I4" s="1" t="inlineStr">
+      <c r="J4" s="1" t="inlineStr">
         <is>
           <t>YES</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t>INSTALL_TRIGGERED</t>
+        </is>
+      </c>
+      <c r="M4" s="1" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="N4" s="1" t="inlineStr">
+        <is>
+          <t>CLEANED</t>
         </is>
       </c>
     </row>
     <row r="5" ht="13.9" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>SW4</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>C8KV</t>
+          <t>C9200</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>10.17.1.12</t>
+          <t>10.17.1.16</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>17.13.1a</t>
+          <t>17.15.4</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>17.15.04c</t>
+          <t>17.15.05</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -764,117 +1169,411 @@
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
+          <t>AUTH_OK</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="H5" s="1" t="inlineStr">
+      <c r="I5" s="1" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="I5" s="1" t="inlineStr">
+      <c r="J5" s="1" t="inlineStr">
         <is>
           <t>YES</t>
+        </is>
+      </c>
+      <c r="K5" s="1" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="L5" s="1" t="inlineStr">
+        <is>
+          <t>INSTALL_TRIGGERED</t>
+        </is>
+      </c>
+      <c r="M5" s="1" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="N5" s="1" t="inlineStr">
+        <is>
+          <t>CLEANED</t>
         </is>
       </c>
     </row>
     <row r="6" ht="13.9" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>C8KV</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>10.17.1.11</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>17.13.1a</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>17.15.04c</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>AUTH_OK</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K6" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L6" s="1" t="inlineStr">
+        <is>
+          <t>NOT_ATTEMPTED</t>
+        </is>
+      </c>
+      <c r="M6" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N6" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="13.9" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>C8KV</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>10.17.1.12</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v/>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>17.15.04c</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>ONLINE</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>AUTH_BAD</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J7" s="1" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K7" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L7" s="1" t="inlineStr">
+        <is>
+          <t>NOT_ATTEMPTED</t>
+        </is>
+      </c>
+      <c r="M7" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N7" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="13.9" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>C8KV</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>10.17.1.13</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>17.13.1a</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>17.12.06</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>ONLINE</t>
         </is>
       </c>
-      <c r="G6" s="1" t="inlineStr">
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>AUTH_OK</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="H6" s="1" t="inlineStr">
+      <c r="I8" s="1" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="I6" s="1" t="inlineStr">
+      <c r="J8" s="1" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
+      <c r="K8" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L8" s="1" t="inlineStr">
+        <is>
+          <t>NOT_ATTEMPTED</t>
+        </is>
+      </c>
+      <c r="M8" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N8" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
-    <row r="7" ht="14.25" customHeight="1"/>
-    <row r="1048575" ht="12.75" customHeight="1"/>
-    <row r="1048576" ht="12.75" customHeight="1"/>
+    <row r="9" ht="14.25" customHeight="1"/>
   </sheetData>
+  <conditionalFormatting sqref="A4:A5">
+    <cfRule type="expression" priority="38" dxfId="31">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" priority="37" dxfId="30">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A2:E3">
-    <cfRule type="expression" priority="23" dxfId="12">
+    <cfRule type="expression" priority="61" dxfId="30">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" priority="24" dxfId="11">
+    <cfRule type="expression" priority="62" dxfId="31">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:E6">
-    <cfRule type="expression" priority="25" dxfId="10">
+  <conditionalFormatting sqref="A6:E8">
+    <cfRule type="expression" priority="64" dxfId="35">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" priority="63" dxfId="34">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" priority="26" dxfId="9">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4:B5">
+    <cfRule type="expression" priority="36" dxfId="31">
       <formula>ISODD(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" priority="35" dxfId="30">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C4:E5">
+    <cfRule type="expression" priority="34" dxfId="31">
+      <formula>ISODD(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" priority="33" dxfId="30">
+      <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F1048576">
-    <cfRule type="cellIs" priority="13" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="52" operator="equal" dxfId="1">
+      <formula>"OFFLINE"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="51" operator="equal" dxfId="0">
       <formula>"ONLINE"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="14" operator="equal" dxfId="0">
-      <formula>"OFFLINE"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="cellIs" priority="10" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="31" operator="equal" dxfId="1">
+      <formula>"AUTH_BAD"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="30" operator="equal" dxfId="0">
+      <formula>"AUTH_OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G1:I1048576">
+    <cfRule type="cellIs" priority="29" operator="equal" dxfId="5">
+      <formula>"N/A"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H1:I1048576">
+    <cfRule type="cellIs" priority="50" operator="equal" dxfId="0">
+      <formula>"YES"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="49" operator="equal" dxfId="1">
+      <formula>"NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H1:K1048576">
+    <cfRule type="cellIs" priority="25" operator="equal" dxfId="5">
       <formula>"UNKNOWN"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1:H1048576">
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+  <conditionalFormatting sqref="J1:J1048576">
+    <cfRule type="cellIs" priority="40" operator="equal" dxfId="1">
+      <formula>"YES"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="39" operator="equal" dxfId="0">
+      <formula>"NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K1:K1048576">
+    <cfRule type="cellIs" priority="28" operator="equal" dxfId="1">
+      <formula>"FAILED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="24" operator="equal" dxfId="5">
       <formula>"N/A"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="0">
-      <formula>"NO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" dxfId="1">
-      <formula>"YES"</formula>
+    <cfRule type="cellIs" priority="27" operator="equal" dxfId="0">
+      <formula>"SUCCESS"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
-      <formula>"NO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
-      <formula>"YES"</formula>
+  <conditionalFormatting sqref="L1:L1048576">
+    <cfRule type="cellIs" priority="20" operator="equal" dxfId="5">
+      <formula>"NOT_ATTEMPTED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="19" operator="equal" dxfId="1">
+      <formula>"CONNECT_ERROR"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="1">
+      <formula>"UNEXPECTED_ERROR"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="1">
+      <formula>"ADD_FAILED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="1">
+      <formula>"ACTIVATE_FAILED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="22" operator="equal" dxfId="0">
+      <formula>"INSTALL_TRIGGERED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="21" operator="equal" dxfId="5">
+      <formula>"ABORTED"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M1:M1048576">
+    <cfRule type="cellIs" priority="16" operator="equal" dxfId="0">
+      <formula>"SUCCESS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="1">
+      <formula>"FAILED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="5">
+      <formula>"COMMIT_FAILED"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M1:N1048576">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="5">
+      <formula>"N/A"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
+      <formula>"UNKNOWN"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N1:N1048576">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="0">
+      <formula>"CLEANED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
+      <formula>"CLEANED_FAILED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+      <formula>"CONNECT_ERROR"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"UNEXPECTED_ERROR"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"NOTHING_TO_CLEAN"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Fully Operational: implemented a GUI with buttons, and error handling for most cases. There are still a couple bugs to solve, and it has only been tested in C9200CXs fully. The GUI looks acceptable, even though some style corrections could be made to make it more attractive. I haven't compiled once at this point, so we also have to test how it works with compiling.
</commit_message>
<xml_diff>
--- a/LAN_Network_Devices.xlsx
+++ b/LAN_Network_Devices.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LAB_NETAUTO001" sheetId="1" state="visible" r:id="rId1"/>
@@ -31,7 +31,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +41,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
         <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
@@ -72,11 +78,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -849,17 +856,17 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Hostname</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>OOBM IP Address</t>
         </is>
@@ -869,7 +876,7 @@
           <t>Current IOS Version</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Recommended IOS Version</t>
         </is>
@@ -936,11 +943,7 @@
           <t>10.17.1.10</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>17.12.1prd9</t>
-        </is>
-      </c>
+      <c r="D2" s="1" t="inlineStr"/>
       <c r="E2" s="1" t="inlineStr">
         <is>
           <t>17.12.02prd9</t>
@@ -948,27 +951,27 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>ONLINE</t>
+          <t>OFFLINE</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>AUTH_OK</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
           <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="I2" s="1" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="inlineStr">
-        <is>
-          <t>YES</t>
         </is>
       </c>
       <c r="K2" s="1" t="inlineStr">
@@ -1082,12 +1085,12 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>17.12.6</t>
+          <t>17.12.5</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>17.12.05</t>
+          <t>17.12.06</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
@@ -1154,12 +1157,12 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>17.15.4</t>
+          <t>17.15.5</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>17.15.05</t>
+          <t>17.15.04</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -1224,11 +1227,7 @@
           <t>10.17.1.11</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>17.13.1a</t>
-        </is>
-      </c>
+      <c r="D6" s="1" t="inlineStr"/>
       <c r="E6" s="1" t="inlineStr">
         <is>
           <t>17.15.04c</t>
@@ -1241,22 +1240,22 @@
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>AUTH_OK</t>
+          <t>AUTH_BAD</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I6" s="1" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J6" s="1" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="K6" s="1" t="inlineStr">
@@ -1296,12 +1295,14 @@
           <t>10.17.1.12</t>
         </is>
       </c>
-      <c r="D7" s="1" t="n">
-        <v/>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>17.13.1a</t>
+        </is>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>17.15.04c</t>
+          <t>17.15.05c</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
@@ -1311,22 +1312,22 @@
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>AUTH_BAD</t>
+          <t>AUTH_OK</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="I7" s="1" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="J7" s="1" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="K7" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Fully Operational: removed the enabling of SCP and RESTCONF from the application functionality. We don't want to be responsible of security issued due to such services being enabled. Therefore, it is up to the user to enable them. Instead, we use a test command to check if devices are online or offline. Fixed a bunch of bugs as well, like the watchdog initialization, timeouts and intervals for RESTCONF status, duplicate call on the Cancel button enabling, ...
</commit_message>
<xml_diff>
--- a/LAN_Network_Devices.xlsx
+++ b/LAN_Network_Devices.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LAB_NETAUTO001" sheetId="1" state="visible" r:id="rId1"/>
@@ -78,224 +78,230 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="50">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
+  <dxfs count="105">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.5998718222602009"/>
         </patternFill>
       </fill>
     </dxf>
@@ -323,6 +329,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="5" tint="0.5998718222602009"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.7998901333658864"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="4" tint="0.5998718222602009"/>
         </patternFill>
       </fill>
@@ -330,6 +350,363 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="4" tint="0.7998901333658864"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.5998718222602009"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.7998901333658864"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.7998901333658864"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.5998718222602009"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.7998901333658864"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.5998718222602009"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="5" tint="0.7998901333658864"/>
         </patternFill>
       </fill>
@@ -368,6 +745,34 @@
           <bgColor theme="4" tint="0.5998718222602009"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <border>
@@ -554,11 +959,6 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -634,7 +1034,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1_2" displayName="Table1_2" ref="A1:N8" headerRowCount="1" totalsRowShown="0" headerRowDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1_2" displayName="Table1_2" ref="A1:N8" headerRowCount="1" totalsRowShown="0" headerRowDxfId="94" headerRowBorderDxfId="95">
   <autoFilter ref="A1:N8"/>
   <tableColumns count="14">
     <tableColumn id="1" name="Hostname"/>
@@ -642,15 +1042,15 @@
     <tableColumn id="3" name="OOBM IP Address"/>
     <tableColumn id="4" name="Current IOS Version"/>
     <tableColumn id="5" name="Recommended IOS Version"/>
-    <tableColumn id="6" name="Status" dataDxfId="48"/>
-    <tableColumn id="10" name="Auth Status" dataDxfId="47"/>
-    <tableColumn id="7" name="Enough Flash Space" dataDxfId="46"/>
-    <tableColumn id="9" name="Update IOS File Present" dataDxfId="45"/>
-    <tableColumn id="8" name="Needs Update" dataDxfId="44"/>
-    <tableColumn id="12" name="Transfer Result" dataDxfId="43"/>
-    <tableColumn id="11" name="Install Status" dataDxfId="42"/>
-    <tableColumn id="13" name="Update Result" dataDxfId="41"/>
-    <tableColumn id="14" name="Cleaned Inactive" dataDxfId="40"/>
+    <tableColumn id="6" name="Status" dataDxfId="104"/>
+    <tableColumn id="10" name="Auth Status" dataDxfId="103"/>
+    <tableColumn id="7" name="Enough Flash Space" dataDxfId="102"/>
+    <tableColumn id="9" name="Update IOS File Present" dataDxfId="101"/>
+    <tableColumn id="8" name="Needs Update" dataDxfId="100"/>
+    <tableColumn id="12" name="Transfer Result" dataDxfId="99"/>
+    <tableColumn id="11" name="Install Status" dataDxfId="98"/>
+    <tableColumn id="13" name="Update Result" dataDxfId="97"/>
+    <tableColumn id="14" name="Cleaned Inactive" dataDxfId="96"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -856,17 +1256,17 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Hostname</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>OOBM IP Address</t>
         </is>
@@ -876,7 +1276,7 @@
           <t>Current IOS Version</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Recommended IOS Version</t>
         </is>
@@ -896,32 +1296,32 @@
           <t>Enough Flash Space</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Update IOS File Present</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Needs Update</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Transfer Result</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Install Status</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Update Result</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>Cleaned Inactive</t>
         </is>
@@ -974,26 +1374,10 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="K2" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L2" s="1" t="inlineStr">
-        <is>
-          <t>NOT_ATTEMPTED</t>
-        </is>
-      </c>
-      <c r="M2" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N2" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="K2" s="1" t="inlineStr"/>
+      <c r="L2" s="1" t="inlineStr"/>
+      <c r="M2" s="1" t="inlineStr"/>
+      <c r="N2" s="1" t="inlineStr"/>
     </row>
     <row r="3" ht="13.9" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
@@ -1046,26 +1430,10 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K3" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L3" s="1" t="inlineStr">
-        <is>
-          <t>NOT_ATTEMPTED</t>
-        </is>
-      </c>
-      <c r="M3" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N3" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="K3" s="1" t="inlineStr"/>
+      <c r="L3" s="1" t="inlineStr"/>
+      <c r="M3" s="1" t="inlineStr"/>
+      <c r="N3" s="1" t="inlineStr"/>
     </row>
     <row r="4" ht="13.9" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
@@ -1083,11 +1451,7 @@
           <t>10.17.1.15</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>17.12.5</t>
-        </is>
-      </c>
+      <c r="D4" s="1" t="inlineStr"/>
       <c r="E4" s="1" t="inlineStr">
         <is>
           <t>17.12.06</t>
@@ -1105,39 +1469,23 @@
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J4" s="1" t="inlineStr">
         <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K4" s="1" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="L4" s="1" t="inlineStr">
-        <is>
-          <t>INSTALL_TRIGGERED</t>
-        </is>
-      </c>
-      <c r="M4" s="1" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="N4" s="1" t="inlineStr">
-        <is>
-          <t>CLEANED</t>
-        </is>
-      </c>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr"/>
+      <c r="L4" s="1" t="inlineStr"/>
+      <c r="M4" s="1" t="inlineStr"/>
+      <c r="N4" s="1" t="inlineStr"/>
     </row>
     <row r="5" ht="13.9" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
@@ -1190,26 +1538,10 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="K5" s="1" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="L5" s="1" t="inlineStr">
-        <is>
-          <t>INSTALL_TRIGGERED</t>
-        </is>
-      </c>
-      <c r="M5" s="1" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="N5" s="1" t="inlineStr">
-        <is>
-          <t>CLEANED</t>
-        </is>
-      </c>
+      <c r="K5" s="1" t="inlineStr"/>
+      <c r="L5" s="1" t="inlineStr"/>
+      <c r="M5" s="1" t="inlineStr"/>
+      <c r="N5" s="1" t="inlineStr"/>
     </row>
     <row r="6" ht="13.9" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
@@ -1258,26 +1590,10 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="K6" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L6" s="1" t="inlineStr">
-        <is>
-          <t>NOT_ATTEMPTED</t>
-        </is>
-      </c>
-      <c r="M6" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N6" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="K6" s="1" t="inlineStr"/>
+      <c r="L6" s="1" t="inlineStr"/>
+      <c r="M6" s="1" t="inlineStr"/>
+      <c r="N6" s="1" t="inlineStr"/>
     </row>
     <row r="7" ht="13.9" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
@@ -1330,26 +1646,10 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="K7" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L7" s="1" t="inlineStr">
-        <is>
-          <t>NOT_ATTEMPTED</t>
-        </is>
-      </c>
-      <c r="M7" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N7" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="K7" s="1" t="inlineStr"/>
+      <c r="L7" s="1" t="inlineStr"/>
+      <c r="M7" s="1" t="inlineStr"/>
+      <c r="N7" s="1" t="inlineStr"/>
     </row>
     <row r="8" ht="13.9" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
@@ -1402,179 +1702,163 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="K8" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L8" s="1" t="inlineStr">
-        <is>
-          <t>NOT_ATTEMPTED</t>
-        </is>
-      </c>
-      <c r="M8" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N8" s="1" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="K8" s="1" t="inlineStr"/>
+      <c r="L8" s="1" t="inlineStr"/>
+      <c r="M8" s="1" t="inlineStr"/>
+      <c r="N8" s="1" t="inlineStr"/>
     </row>
     <row r="9" ht="14.25" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="A4:A5">
-    <cfRule type="expression" priority="38" dxfId="31">
+    <cfRule type="expression" priority="44" dxfId="31">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" priority="45" dxfId="30">
       <formula>ISODD(ROW())</formula>
-    </cfRule>
-    <cfRule type="expression" priority="37" dxfId="30">
-      <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:E3">
-    <cfRule type="expression" priority="61" dxfId="30">
+    <cfRule type="expression" priority="68" dxfId="31">
       <formula>ISEVEN(ROW())</formula>
     </cfRule>
-    <cfRule type="expression" priority="62" dxfId="31">
+    <cfRule type="expression" priority="69" dxfId="30">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A6:E8">
-    <cfRule type="expression" priority="64" dxfId="35">
+    <cfRule type="expression" priority="70" dxfId="35">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" priority="71" dxfId="34">
       <formula>ISODD(ROW())</formula>
-    </cfRule>
-    <cfRule type="expression" priority="63" dxfId="34">
-      <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:B5">
-    <cfRule type="expression" priority="36" dxfId="31">
+    <cfRule type="expression" priority="42" dxfId="31">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" priority="43" dxfId="30">
       <formula>ISODD(ROW())</formula>
-    </cfRule>
-    <cfRule type="expression" priority="35" dxfId="30">
-      <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:E5">
-    <cfRule type="expression" priority="34" dxfId="31">
+    <cfRule type="expression" priority="40" dxfId="31">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+    <cfRule type="expression" priority="41" dxfId="30">
       <formula>ISODD(ROW())</formula>
-    </cfRule>
-    <cfRule type="expression" priority="33" dxfId="30">
-      <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F1048576">
-    <cfRule type="cellIs" priority="52" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="58" operator="equal" dxfId="0">
+      <formula>"ONLINE"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="59" operator="equal" dxfId="1">
       <formula>"OFFLINE"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="51" operator="equal" dxfId="0">
-      <formula>"ONLINE"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="cellIs" priority="31" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="37" operator="equal" dxfId="0">
+      <formula>"AUTH_OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="38" operator="equal" dxfId="1">
       <formula>"AUTH_BAD"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="30" operator="equal" dxfId="0">
-      <formula>"AUTH_OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:I1048576">
-    <cfRule type="cellIs" priority="29" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="36" operator="equal" dxfId="5">
       <formula>"N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1048576">
-    <cfRule type="cellIs" priority="50" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="56" operator="equal" dxfId="1">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="57" operator="equal" dxfId="0">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="49" operator="equal" dxfId="1">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:K1048576">
-    <cfRule type="cellIs" priority="25" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="32" operator="equal" dxfId="5">
       <formula>"UNKNOWN"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="cellIs" priority="40" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="46" operator="equal" dxfId="0">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="47" operator="equal" dxfId="1">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="39" operator="equal" dxfId="0">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:K1048576">
-    <cfRule type="cellIs" priority="28" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="31" operator="equal" dxfId="5">
+      <formula>"N/A"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="34" operator="equal" dxfId="0">
+      <formula>"SUCCESS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="35" operator="equal" dxfId="1">
       <formula>"FAILED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="24" operator="equal" dxfId="5">
-      <formula>"N/A"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="27" operator="equal" dxfId="0">
-      <formula>"SUCCESS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L1:L1048576">
-    <cfRule type="cellIs" priority="20" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="17" operator="equal" dxfId="1">
+      <formula>"ACTIVATE_FAILED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="1">
+      <formula>"ADD_FAILED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="25" operator="equal" dxfId="1">
+      <formula>"UNEXPECTED_ERROR"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="26" operator="equal" dxfId="1">
+      <formula>"CONNECT_ERROR"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="27" operator="equal" dxfId="5">
       <formula>"NOT_ATTEMPTED"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="19" operator="equal" dxfId="1">
-      <formula>"CONNECT_ERROR"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="18" operator="equal" dxfId="1">
-      <formula>"UNEXPECTED_ERROR"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="1">
-      <formula>"ADD_FAILED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" dxfId="1">
-      <formula>"ACTIVATE_FAILED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="22" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="28" operator="equal" dxfId="5">
+      <formula>"ABORTED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="29" operator="equal" dxfId="0">
       <formula>"INSTALL_TRIGGERED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="21" operator="equal" dxfId="5">
-      <formula>"ABORTED"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M1:M1048576">
-    <cfRule type="cellIs" priority="16" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="16" operator="equal" dxfId="5">
+      <formula>"COMMIT_FAILED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="20" operator="equal" dxfId="1">
+      <formula>"FAILED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="23" operator="equal" dxfId="0">
       <formula>"SUCCESS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" dxfId="1">
-      <formula>"FAILED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="5">
-      <formula>"COMMIT_FAILED"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M1:N1048576">
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="5">
+      <formula>"UNKNOWN"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="5">
       <formula>"N/A"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
-      <formula>"UNKNOWN"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:N1048576">
     <cfRule type="cellIs" priority="8" operator="equal" dxfId="0">
+      <formula>"NOTHING_TO_CLEAN"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="1">
+      <formula>"UNEXPECTED_ERROR"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="1">
+      <formula>"CONNECT_ERROR"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="1">
+      <formula>"CLEANED_FAILED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="0">
       <formula>"CLEANED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
-      <formula>"CLEANED_FAILED"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
-      <formula>"CONNECT_ERROR"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
-      <formula>"UNEXPECTED_ERROR"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"NOTHING_TO_CLEAN"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Fully Operational: corrected a few details in the comments, and wrap it up for this version, which does not include the Command Pusher mode neither mode election
</commit_message>
<xml_diff>
--- a/LAN_Network_Devices.xlsx
+++ b/LAN_Network_Devices.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LAB_NETAUTO001" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LAB_NETAUTO001" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -1374,10 +1374,26 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="K2" s="1" t="inlineStr"/>
-      <c r="L2" s="1" t="inlineStr"/>
-      <c r="M2" s="1" t="inlineStr"/>
-      <c r="N2" s="1" t="inlineStr"/>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>NOT_ATTEMPTED</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N2" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="13.9" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
@@ -1430,10 +1446,26 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="K3" s="1" t="inlineStr"/>
-      <c r="L3" s="1" t="inlineStr"/>
-      <c r="M3" s="1" t="inlineStr"/>
-      <c r="N3" s="1" t="inlineStr"/>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>NOT_ATTEMPTED</t>
+        </is>
+      </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="13.9" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
@@ -1451,7 +1483,11 @@
           <t>10.17.1.15</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr"/>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>17.12.5</t>
+        </is>
+      </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
           <t>17.12.06</t>
@@ -1469,23 +1505,39 @@
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="J4" s="1" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="K4" s="1" t="inlineStr"/>
-      <c r="L4" s="1" t="inlineStr"/>
-      <c r="M4" s="1" t="inlineStr"/>
-      <c r="N4" s="1" t="inlineStr"/>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t>INSTALL_TRIGGERED</t>
+        </is>
+      </c>
+      <c r="M4" s="1" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="N4" s="1" t="inlineStr">
+        <is>
+          <t>CLEANED</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="13.9" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
@@ -1538,10 +1590,26 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="K5" s="1" t="inlineStr"/>
-      <c r="L5" s="1" t="inlineStr"/>
-      <c r="M5" s="1" t="inlineStr"/>
-      <c r="N5" s="1" t="inlineStr"/>
+      <c r="K5" s="1" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="L5" s="1" t="inlineStr">
+        <is>
+          <t>INSTALL_TRIGGERED</t>
+        </is>
+      </c>
+      <c r="M5" s="1" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="N5" s="1" t="inlineStr">
+        <is>
+          <t>CLEANED</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="13.9" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
@@ -1590,10 +1658,26 @@
           <t>UNKNOWN</t>
         </is>
       </c>
-      <c r="K6" s="1" t="inlineStr"/>
-      <c r="L6" s="1" t="inlineStr"/>
-      <c r="M6" s="1" t="inlineStr"/>
-      <c r="N6" s="1" t="inlineStr"/>
+      <c r="K6" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L6" s="1" t="inlineStr">
+        <is>
+          <t>NOT_ATTEMPTED</t>
+        </is>
+      </c>
+      <c r="M6" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N6" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="13.9" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
@@ -1646,10 +1730,26 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="K7" s="1" t="inlineStr"/>
-      <c r="L7" s="1" t="inlineStr"/>
-      <c r="M7" s="1" t="inlineStr"/>
-      <c r="N7" s="1" t="inlineStr"/>
+      <c r="K7" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L7" s="1" t="inlineStr">
+        <is>
+          <t>NOT_ATTEMPTED</t>
+        </is>
+      </c>
+      <c r="M7" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N7" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="13.9" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
@@ -1702,10 +1802,26 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="K8" s="1" t="inlineStr"/>
-      <c r="L8" s="1" t="inlineStr"/>
-      <c r="M8" s="1" t="inlineStr"/>
-      <c r="N8" s="1" t="inlineStr"/>
+      <c r="K8" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L8" s="1" t="inlineStr">
+        <is>
+          <t>NOT_ATTEMPTED</t>
+        </is>
+      </c>
+      <c r="M8" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N8" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1"/>
   </sheetData>

</xml_diff>